<commit_message>
add evidence gap map
update evidence table (RoB domains)
</commit_message>
<xml_diff>
--- a/data/Evidence_Table.xlsx
+++ b/data/Evidence_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saramanaye/Documents/GitHub/cancer_nutrition_evidence_review/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07ACB602-DE58-8244-A470-3C1C96C8AB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805090BA-5B35-1647-9E31-AA6375ED02D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Table" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="319">
   <si>
     <t>Year</t>
   </si>
@@ -645,9 +645,6 @@
     <t>Control group- received usual care</t>
   </si>
   <si>
-    <t>6 months</t>
-  </si>
-  <si>
     <t>Exercise - 41% were adherent to aerobic exercise and 26% were adherent to resistance training</t>
   </si>
   <si>
@@ -669,9 +666,6 @@
   </si>
   <si>
     <t>Control group -received standard care, following hospital's  ERAS  protocol</t>
-  </si>
-  <si>
-    <t>14.2 ± 3.6 weeks</t>
   </si>
   <si>
     <t>The study relied on self-reported logs rather than wearable device data and had a small sample size. It also lacked detailed daily nutritional intake data and was conducted at a single center, which may limit the generalizability of the findings</t>
@@ -750,9 +744,6 @@
   </si>
   <si>
     <t>3-6 weeks</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92 (±33) days</t>
   </si>
   <si>
     <t>17 days</t>
@@ -917,9 +908,6 @@
 92% for psychological counseling</t>
   </si>
   <si>
-    <t>The study faced selection bias from excluding unwilling participants and variability in chemotherapy regimens which may affect generalizability. Additionally, the short follow-up period meant long-term outcomes like progression-free and overall survival were not assessed</t>
-  </si>
-  <si>
     <t>3 weeks</t>
   </si>
   <si>
@@ -971,17 +959,10 @@
     <t>Quality of Recovery-15 (QoR-15)</t>
   </si>
   <si>
-    <t>Performance bias
-Detection bias</t>
-  </si>
-  <si>
     <t>Feasibility</t>
   </si>
   <si>
     <t>Postoperative complications</t>
-  </si>
-  <si>
-    <t>Performance bias</t>
   </si>
   <si>
     <t>Functional capacity</t>
@@ -1003,14 +984,6 @@
 Nutritional status</t>
   </si>
   <si>
-    <t>Selection bias
-Performance bias</t>
-  </si>
-  <si>
-    <t>Performance bias
-Attrition bias</t>
-  </si>
-  <si>
     <t>30-day postoperative Comprehensive Complication Index (CCI)</t>
   </si>
   <si>
@@ -1019,12 +992,6 @@
   </si>
   <si>
     <t>Randomized Controlled Feasibility Trial</t>
-  </si>
-  <si>
-    <t>Performance bias
-Detection bias
-Reporting bias
-Attrition bias</t>
   </si>
   <si>
     <t xml:space="preserve">Some concerns </t>
@@ -1146,10 +1113,6 @@
     <t>For older patients, optimal delivery requires a synergistic approach, as the sources demonstrate that exercise alone is insufficient to increase skeletal muscle mass during chemotherapy. The nutrition component must specifically include leucine-rich amino acids to overcome the anabolic resistance common in the elderly, effectively stimulating muscle protein synthesis. To address the low compliance seen in this trial, delivery should involve a multidisciplinary team providing continuous monitoring and patient interviews. Furthermore, exercise should be individually tailored in intensity to accommodate the variable physical capacities of older adults, which can enhance overall adherence and clinical outcomes.</t>
   </si>
   <si>
-    <t>Performance bias
-Unclear Detection bias</t>
-  </si>
-  <si>
     <t>a synergistic multidisciplinary approach is required where resistance training provides the mechanical stimulus and targeted nutrition - specifically leucine-rich amino acids or HMB which overcomes anabolic resistance in older adults. The  nutrition component must be carefully monitored to ensure high adherence, as the preservation of lean body mass is significantly greater in patients who strictly follow both the exercise and supplement protocols. To be most effective, programs should be risk-adapted, focusing on vulnerable populations (such as women or those with low baseline muscle mass) who demonstrate the highest potential for measurable improvement. Furthermore, a duration longer than the average 17 days may be necessary to build a durable physiological reserve that can withstand the intense catabolic stress of major surgery</t>
   </si>
   <si>
@@ -1188,13 +1151,61 @@
   </si>
   <si>
     <t>multimodal prehabilitation should prioritize high-risk, sedentary patients, who are significantly more likely to see meaningful improvements in functional capacity (most significant benefits were seen in previously inactive and sedentary patients, particularly women, who were 7.07 times more likely to improve functional capacity through prehabilitation). Effective programs must integrate aerobic and resistance exercise with nutritional support, specifically timing protein intake within the "anabolic window" for maximum benefit. To outperform standard home-based programs, practitioners should consider increased exercise intensity or a higher frequency of supervised sessions. Finally, involving qualified professionals for supervision is essential to promote patient confidence and ensure adherence to recommended clinical goals</t>
+  </si>
+  <si>
+    <t>The study faced selection bias from excluding unwilling participants and variability in chemotherapy regimens which may affect generalizability. Additionally, the short follow-up period meant long-term outcomes like progression-free and overall survival were not assessed. The use of quasi-randomization (odd-even method) place the study at a high risk for bias despite the blinding of outcome assessors</t>
+  </si>
+  <si>
+    <t>For the duration of NACT</t>
+  </si>
+  <si>
+    <t>32 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92 days</t>
+  </si>
+  <si>
+    <t>14.2 weeks</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Attrition bias (Domain 3)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Attrition bias  (Domain 3)</t>
+  </si>
+  <si>
+    <t>Selection bias (Domain 1)
+Performance bias (Domain 2)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Unclear Detection bias (Domain 4)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Detection bias  (Domain 4)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Unclear Detection bias  (Domain 4)</t>
+  </si>
+  <si>
+    <t>Performance bias (Domain 2)
+Detection bias  (Domain 4)
+Reporting bias  (Domain 5)
+Attrition bias (Domain 3)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1277,12 +1288,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color rgb="FF222222"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
@@ -1350,7 +1355,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1359,7 +1363,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1698,7 +1703,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12.5" style="3" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" customWidth="1"/>
     <col min="4" max="4" width="37" style="6" customWidth="1"/>
     <col min="5" max="6" width="22.5" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
@@ -1728,7 +1733,7 @@
         <v>6</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -1746,31 +1751,31 @@
         <v>1</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>93</v>
@@ -1782,40 +1787,40 @@
         <v>2</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>94</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>95</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="153">
@@ -1850,7 +1855,7 @@
         <v>4</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>4</v>
@@ -1859,34 +1864,34 @@
         <v>4</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>115</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q2" s="6" t="s">
         <v>98</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="S2" s="4" t="s">
         <v>90</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V2" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X2" s="4" t="s">
         <v>115</v>
@@ -1895,22 +1900,22 @@
         <v>115</v>
       </c>
       <c r="Z2" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="AA2" s="4" t="s">
         <v>99</v>
       </c>
       <c r="AB2" s="4" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="AC2" s="4" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD2" s="4" t="s">
         <v>91</v>
       </c>
       <c r="AE2" s="4" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="255">
@@ -1933,7 +1938,7 @@
         <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>101</v>
@@ -1945,7 +1950,7 @@
         <v>4</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>4</v>
@@ -1954,10 +1959,10 @@
         <v>4</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P3" s="6" t="s">
         <v>4</v>
@@ -1966,22 +1971,22 @@
         <v>104</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>151</v>
+        <v>308</v>
       </c>
       <c r="S3" s="4" t="s">
         <v>102</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W3" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X3" s="4" t="s">
         <v>115</v>
@@ -1996,16 +2001,16 @@
         <v>105</v>
       </c>
       <c r="AB3" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC3" s="4" t="s">
-        <v>265</v>
+        <v>313</v>
       </c>
       <c r="AD3" s="4" t="s">
         <v>106</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="221">
@@ -2028,7 +2033,7 @@
         <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>108</v>
@@ -2040,7 +2045,7 @@
         <v>4</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>4</v>
@@ -2049,10 +2054,10 @@
         <v>4</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>4</v>
@@ -2061,28 +2066,28 @@
         <v>109</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X4" s="6" t="s">
         <v>115</v>
       </c>
       <c r="Y4" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z4" s="6" t="s">
         <v>115</v>
@@ -2091,16 +2096,16 @@
         <v>110</v>
       </c>
       <c r="AB4" s="6" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC4" s="6" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD4" s="6" t="s">
         <v>111</v>
       </c>
       <c r="AE4" s="6" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:31" s="5" customFormat="1" ht="153">
@@ -2123,7 +2128,7 @@
         <v>113</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>112</v>
@@ -2132,7 +2137,7 @@
         <v>4</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>4</v>
@@ -2147,7 +2152,7 @@
         <v>4</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>4</v>
@@ -2156,28 +2161,28 @@
         <v>114</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="S5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W5" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X5" s="4" t="s">
         <v>115</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z5" s="4" t="s">
         <v>115</v>
@@ -2186,16 +2191,16 @@
         <v>115</v>
       </c>
       <c r="AB5" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC5" s="4" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD5" s="4" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="AE5" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:31" s="3" customFormat="1" ht="204">
@@ -2212,13 +2217,13 @@
         <v>18</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>117</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>20</v>
@@ -2230,7 +2235,7 @@
         <v>4</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>4</v>
@@ -2257,10 +2262,10 @@
         <v>19</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V6" s="4" t="s">
         <v>115</v>
@@ -2269,10 +2274,10 @@
         <v>115</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z6" s="4" t="s">
         <v>115</v>
@@ -2281,16 +2286,16 @@
         <v>119</v>
       </c>
       <c r="AB6" s="4" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="AC6" s="4" t="s">
-        <v>269</v>
+        <v>318</v>
       </c>
       <c r="AD6" s="4" t="s">
         <v>120</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="170">
@@ -2313,7 +2318,7 @@
         <v>127</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>23</v>
@@ -2325,7 +2330,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>4</v>
@@ -2352,22 +2357,22 @@
         <v>24</v>
       </c>
       <c r="T7" s="8" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="U7" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V7" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W7" s="8" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X7" s="8" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Y7" s="8" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z7" s="8" t="s">
         <v>115</v>
@@ -2376,16 +2381,16 @@
         <v>129</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC7" s="8" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD7" s="4" t="s">
         <v>130</v>
       </c>
       <c r="AE7" s="4" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:31" s="3" customFormat="1" ht="187">
@@ -2408,7 +2413,7 @@
         <v>131</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>28</v>
@@ -2432,7 +2437,7 @@
         <v>4</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P8" s="5" t="s">
         <v>4</v>
@@ -2441,46 +2446,46 @@
         <v>132</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>188</v>
+        <v>309</v>
       </c>
       <c r="S8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X8" s="4" t="s">
         <v>115</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="AA8" s="4" t="s">
         <v>115</v>
       </c>
       <c r="AB8" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC8" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD8" s="4" t="s">
         <v>133</v>
       </c>
       <c r="AE8" s="4" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:31" ht="204">
@@ -2527,7 +2532,7 @@
         <v>4</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>4</v>
@@ -2542,40 +2547,40 @@
         <v>44</v>
       </c>
       <c r="T9" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W9" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X9" s="4" t="s">
         <v>115</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z9" s="4" t="s">
         <v>115</v>
       </c>
       <c r="AA9" s="4" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="AB9" s="4" t="s">
         <v>116</v>
       </c>
       <c r="AC9" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD9" s="4" t="s">
         <v>136</v>
       </c>
       <c r="AE9" s="4" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:31" s="3" customFormat="1" ht="204">
@@ -2598,7 +2603,7 @@
         <v>138</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>47</v>
@@ -2625,7 +2630,7 @@
         <v>4</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>139</v>
@@ -2637,16 +2642,16 @@
         <v>48</v>
       </c>
       <c r="T10" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V10" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W10" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X10" s="4" t="s">
         <v>115</v>
@@ -2664,13 +2669,13 @@
         <v>116</v>
       </c>
       <c r="AC10" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD10" s="4" t="s">
         <v>140</v>
       </c>
       <c r="AE10" s="4" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:31" ht="238">
@@ -2693,7 +2698,7 @@
         <v>141</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>49</v>
@@ -2705,7 +2710,7 @@
         <v>4</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>4</v>
@@ -2714,10 +2719,10 @@
         <v>4</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>4</v>
@@ -2732,40 +2737,40 @@
         <v>50</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W11" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X11" s="4" t="s">
         <v>115</v>
       </c>
       <c r="Y11" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z11" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="AA11" s="20">
+      <c r="AA11" s="19">
         <v>0.83299999999999996</v>
       </c>
       <c r="AB11" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC11" s="4" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD11" s="4" t="s">
         <v>145</v>
       </c>
       <c r="AE11" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:31" ht="187">
@@ -2788,7 +2793,7 @@
         <v>146</v>
       </c>
       <c r="G12" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>52</v>
@@ -2821,22 +2826,22 @@
         <v>147</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="T12" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W12" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X12" s="4" t="s">
         <v>115</v>
@@ -2851,16 +2856,16 @@
         <v>115</v>
       </c>
       <c r="AB12" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC12" s="4" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD12" s="4" t="s">
         <v>148</v>
       </c>
       <c r="AE12" s="4" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="221">
@@ -2883,7 +2888,7 @@
         <v>149</v>
       </c>
       <c r="G13" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>54</v>
@@ -2895,7 +2900,7 @@
         <v>4</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>4</v>
@@ -2904,13 +2909,13 @@
         <v>4</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>4</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q13" s="6" t="s">
         <v>150</v>
@@ -2919,22 +2924,22 @@
         <v>151</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="T13" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V13" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W13" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y13" s="4" t="s">
         <v>115</v>
@@ -2946,16 +2951,16 @@
         <v>152</v>
       </c>
       <c r="AB13" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC13" s="4" t="s">
-        <v>254</v>
+        <v>316</v>
       </c>
       <c r="AD13" s="4" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="AE13" s="5" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="170">
@@ -2978,7 +2983,7 @@
         <v>153</v>
       </c>
       <c r="G14" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>57</v>
@@ -2990,7 +2995,7 @@
         <v>4</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>115</v>
@@ -3011,16 +3016,16 @@
         <v>154</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>155</v>
+        <v>307</v>
       </c>
       <c r="S14" s="4" t="s">
         <v>58</v>
       </c>
       <c r="T14" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V14" s="4" t="s">
         <v>115</v>
@@ -3029,28 +3034,28 @@
         <v>115</v>
       </c>
       <c r="X14" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Y14" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z14" s="4" t="s">
         <v>115</v>
       </c>
       <c r="AA14" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AB14" s="4" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="AC14" s="4" t="s">
-        <v>254</v>
+        <v>316</v>
       </c>
       <c r="AD14" s="4" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="AE14" s="4" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="204">
@@ -3070,10 +3075,10 @@
         <v>25</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G15" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>60</v>
@@ -3103,49 +3108,49 @@
         <v>4</v>
       </c>
       <c r="Q15" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="R15" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="R15" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="S15" s="4" t="s">
         <v>61</v>
       </c>
       <c r="T15" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="U15" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V15" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W15" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X15" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y15" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z15" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="AA15" s="21">
+      <c r="AA15" s="20">
         <v>0.873</v>
       </c>
       <c r="AB15" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AC15" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD15" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AE15" s="4" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="204">
@@ -3165,10 +3170,10 @@
         <v>25</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G16" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>62</v>
@@ -3180,7 +3185,7 @@
         <v>4</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L16" s="6" t="s">
         <v>115</v>
@@ -3198,49 +3203,49 @@
         <v>4</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>163</v>
+        <v>310</v>
       </c>
       <c r="S16" s="4" t="s">
         <v>63</v>
       </c>
       <c r="T16" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V16" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z16" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="AA16" s="20">
+        <v>241</v>
+      </c>
+      <c r="AA16" s="19">
         <v>0.84399999999999997</v>
       </c>
       <c r="AB16" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AC16" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD16" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AE16" s="4" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="170">
@@ -3260,10 +3265,10 @@
         <v>25</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G17" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>65</v>
@@ -3275,7 +3280,7 @@
         <v>4</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L17" s="9" t="s">
         <v>4</v>
@@ -3290,10 +3295,10 @@
         <v>4</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="R17" s="9" t="s">
         <v>135</v>
@@ -3302,19 +3307,19 @@
         <v>66</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="U17" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X17" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y17" s="4" t="s">
         <v>115</v>
@@ -3323,19 +3328,19 @@
         <v>115</v>
       </c>
       <c r="AA17" s="4" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="AB17" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC17" s="4" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="AD17" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="AE17" s="4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="1:31" ht="170">
@@ -3355,10 +3360,10 @@
         <v>25</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G18" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>68</v>
@@ -3370,7 +3375,7 @@
         <v>4</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L18" s="4" t="s">
         <v>4</v>
@@ -3379,58 +3384,58 @@
         <v>4</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R18" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S18" s="4" t="s">
         <v>69</v>
       </c>
       <c r="T18" s="4" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="U18" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V18" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W18" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X18" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y18" s="4" t="s">
         <v>115</v>
       </c>
       <c r="Z18" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="AA18" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="AB18" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="AC18" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="AD18" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="AB18" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="AC18" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="AD18" s="4" t="s">
-        <v>172</v>
-      </c>
       <c r="AE18" s="4" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="153">
@@ -3450,10 +3455,10 @@
         <v>25</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G19" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>71</v>
@@ -3465,7 +3470,7 @@
         <v>4</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L19" s="4" t="s">
         <v>4</v>
@@ -3474,37 +3479,37 @@
         <v>115</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="S19" s="4" t="s">
         <v>72</v>
       </c>
       <c r="T19" s="4" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="U19" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="V19" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W19" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X19" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y19" s="4" t="s">
         <v>115</v>
@@ -3513,19 +3518,19 @@
         <v>115</v>
       </c>
       <c r="AA19" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AB19" s="4" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="AC19" s="4" t="s">
-        <v>254</v>
+        <v>316</v>
       </c>
       <c r="AD19" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AE19" s="4" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20" spans="1:31" ht="204">
@@ -3545,10 +3550,10 @@
         <v>25</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>75</v>
@@ -3557,7 +3562,7 @@
         <v>4</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>4</v>
@@ -3572,13 +3577,13 @@
         <v>4</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>4</v>
       </c>
       <c r="Q20" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="R20" s="6" t="s">
         <v>135</v>
@@ -3587,13 +3592,13 @@
         <v>74</v>
       </c>
       <c r="T20" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U20" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V20" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W20" s="4" t="s">
         <v>115</v>
@@ -3602,7 +3607,7 @@
         <v>115</v>
       </c>
       <c r="Y20" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Z20" s="4" t="s">
         <v>115</v>
@@ -3614,13 +3619,13 @@
         <v>3</v>
       </c>
       <c r="AC20" s="4" t="s">
-        <v>254</v>
+        <v>316</v>
       </c>
       <c r="AD20" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AE20" s="4" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="170">
@@ -3640,10 +3645,10 @@
         <v>25</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G21" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>77</v>
@@ -3652,7 +3657,7 @@
         <v>4</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>4</v>
@@ -3667,31 +3672,31 @@
         <v>4</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P21" s="6" t="s">
         <v>4</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="S21" s="4" t="s">
         <v>78</v>
       </c>
       <c r="T21" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V21" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="W21" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X21" s="4" t="s">
         <v>115</v>
@@ -3703,19 +3708,19 @@
         <v>115</v>
       </c>
       <c r="AA21" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AB21" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="AC21" s="4" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="AD21" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="AE21" s="4" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
     </row>
     <row r="22" spans="1:31" s="3" customFormat="1" ht="204">
@@ -3735,7 +3740,7 @@
         <v>81</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>126</v>
@@ -3750,37 +3755,37 @@
         <v>4</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="M22" s="5" t="s">
         <v>4</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P22" s="5" t="s">
         <v>4</v>
       </c>
       <c r="Q22" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="R22" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="S22" s="4" t="s">
         <v>83</v>
       </c>
       <c r="T22" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="U22" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V22" s="4" t="s">
         <v>115</v>
@@ -3789,28 +3794,28 @@
         <v>115</v>
       </c>
       <c r="X22" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Y22" s="4" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="Z22" s="4" t="s">
         <v>115</v>
       </c>
       <c r="AA22" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="AB22" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AC22" s="4" t="s">
-        <v>257</v>
+        <v>311</v>
       </c>
       <c r="AD22" s="5" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="AE22" s="4" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="221">
@@ -3827,13 +3832,13 @@
         <v>85</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>86</v>
@@ -3857,34 +3862,34 @@
         <v>4</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="P23" s="5" t="s">
         <v>4</v>
       </c>
       <c r="Q23" s="5" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="R23" s="5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="S23" s="4" t="s">
         <v>87</v>
       </c>
       <c r="T23" s="4" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="U23" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="V23" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W23" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X23" s="4" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="Y23" s="4" t="s">
         <v>115</v>
@@ -3893,19 +3898,19 @@
         <v>115</v>
       </c>
       <c r="AA23" s="4" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="AB23" s="4" t="s">
         <v>3</v>
       </c>
       <c r="AC23" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="AD23" s="4" t="s">
-        <v>236</v>
+        <v>314</v>
+      </c>
+      <c r="AD23" s="5" t="s">
+        <v>306</v>
       </c>
       <c r="AE23" s="4" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="221">
@@ -3925,82 +3930,82 @@
         <v>25</v>
       </c>
       <c r="F24" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J24" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="K24" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="L24" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="M24" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="N24" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="O24" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="P24" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q24" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="R24" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="S24" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="T24" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="U24" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="V24" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="W24" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="X24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="Y24" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="AA24" s="4" t="s">
         <v>223</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="J24" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="K24" s="22" t="s">
-        <v>244</v>
-      </c>
-      <c r="L24" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="M24" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="N24" s="22" t="s">
-        <v>244</v>
-      </c>
-      <c r="O24" s="22" t="s">
-        <v>244</v>
-      </c>
-      <c r="P24" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q24" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="R24" s="11" t="s">
-        <v>186</v>
-      </c>
-      <c r="S24" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="T24" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="U24" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="V24" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="W24" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="X24" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="Y24" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="Z24" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="AA24" s="4" t="s">
-        <v>226</v>
       </c>
       <c r="AB24" s="6" t="s">
         <v>3</v>
       </c>
       <c r="AC24" s="4" t="s">
-        <v>265</v>
+        <v>312</v>
       </c>
       <c r="AD24" s="4" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AE24" s="4" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="25" spans="1:31" s="3" customFormat="1" ht="221">
@@ -4008,7 +4013,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C25" s="3">
         <v>2022</v>
@@ -4017,85 +4022,85 @@
         <v>121</v>
       </c>
       <c r="E25" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="P25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q25" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="S25" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="T25" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="U25" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="V25" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="W25" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="X25" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="Y25" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z25" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="AA25" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="F25" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="H25" s="4" t="s">
+      <c r="AB25" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC25" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="AD25" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="I25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K25" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="L25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="N25" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="O25" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="P25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q25" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="R25" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="S25" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="T25" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="U25" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="V25" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="W25" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="X25" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="Y25" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="Z25" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="AA25" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="AB25" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="AC25" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="AD25" s="4" t="s">
-        <v>222</v>
-      </c>
       <c r="AE25" s="4" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:31" s="3" customFormat="1" ht="272">
@@ -4115,87 +4120,87 @@
         <v>25</v>
       </c>
       <c r="F26" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="N26" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="O26" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="P26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q26" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="R26" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="S26" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="T26" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U26" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="V26" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="W26" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="X26" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="Y26" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="Z26" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="AA26" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H26" s="5" t="s">
+      <c r="AB26" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC26" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AD26" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="I26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="N26" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="O26" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="P26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q26" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="R26" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="S26" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="T26" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="U26" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="V26" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="W26" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="X26" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="Y26" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="Z26" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="AA26" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="AB26" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="AC26" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="AD26" s="4" t="s">
-        <v>216</v>
-      </c>
       <c r="AE26" s="4" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="27" spans="1:31">
       <c r="A27" s="3"/>
-      <c r="D27" s="19"/>
+      <c r="D27" s="18"/>
       <c r="Q27"/>
     </row>
     <row r="28" spans="1:31">
@@ -4203,57 +4208,63 @@
     </row>
     <row r="29" spans="1:31" ht="18">
       <c r="D29" s="8"/>
-      <c r="Q29" s="23"/>
+      <c r="Q29" s="22"/>
     </row>
     <row r="30" spans="1:31" ht="18">
       <c r="D30" s="8"/>
-      <c r="Q30" s="23"/>
+      <c r="Q30" s="22"/>
     </row>
     <row r="31" spans="1:31" ht="18">
       <c r="D31" s="8"/>
-      <c r="Q31" s="23"/>
+      <c r="Q31" s="22"/>
     </row>
     <row r="32" spans="1:31" ht="18">
       <c r="D32" s="8"/>
-      <c r="Q32" s="23"/>
-    </row>
-    <row r="33" spans="4:4">
+      <c r="Q32" s="22"/>
+    </row>
+    <row r="33" spans="3:4">
       <c r="D33" s="8"/>
     </row>
-    <row r="34" spans="4:4" ht="20">
-      <c r="D34" s="18"/>
-    </row>
-    <row r="35" spans="4:4">
-      <c r="D35" s="8"/>
-    </row>
-    <row r="36" spans="4:4">
-      <c r="D36" s="8"/>
-    </row>
-    <row r="37" spans="4:4">
-      <c r="D37" s="8"/>
-    </row>
-    <row r="38" spans="4:4">
-      <c r="D38" s="8"/>
-    </row>
-    <row r="39" spans="4:4">
-      <c r="D39" s="8"/>
-    </row>
-    <row r="40" spans="4:4">
+    <row r="34" spans="3:4">
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="3:4">
+      <c r="C35" s="1"/>
+      <c r="D35" s="23"/>
+    </row>
+    <row r="36" spans="3:4">
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="3:4">
+      <c r="C37" s="1"/>
+      <c r="D37" s="23"/>
+    </row>
+    <row r="38" spans="3:4">
+      <c r="C38" s="1"/>
+      <c r="D38" s="23"/>
+    </row>
+    <row r="39" spans="3:4">
+      <c r="C39" s="1"/>
+      <c r="D39" s="23"/>
+    </row>
+    <row r="40" spans="3:4">
       <c r="D40" s="8"/>
     </row>
-    <row r="41" spans="4:4">
+    <row r="41" spans="3:4">
       <c r="D41" s="8"/>
     </row>
-    <row r="42" spans="4:4">
+    <row r="42" spans="3:4">
       <c r="D42" s="8"/>
     </row>
-    <row r="43" spans="4:4">
+    <row r="43" spans="3:4">
       <c r="D43" s="8"/>
     </row>
-    <row r="44" spans="4:4">
+    <row r="44" spans="3:4">
       <c r="D44" s="4"/>
     </row>
-    <row r="45" spans="4:4">
+    <row r="45" spans="3:4">
       <c r="D45" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sample size chart updated
</commit_message>
<xml_diff>
--- a/data/Evidence_Table.xlsx
+++ b/data/Evidence_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saramanaye/Documents/GitHub/cancer_nutrition_evidence_review/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FAA694-0EDC-A544-AAAC-9BAFD87591F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BF9A19-CD80-8D40-AD89-B252DEBFB24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="14600" windowHeight="16140" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Table" sheetId="1" r:id="rId1"/>
@@ -327,10 +327,6 @@
 3. Psychology - 60-minute session with a psychology-trained researcher for anxiety reduction + personalized relaxation techniques (visualization and breathing exercises) practiced at home 2-3 times/week using audio tracks</t>
   </si>
   <si>
-    <t>PREHAB+ - 41 (4)
-REHAB - 32  (6)</t>
-  </si>
-  <si>
     <t>REHAB group- received standard post-surgical rehabilitation</t>
   </si>
   <si>
@@ -370,10 +366,6 @@
     <t>Not reported</t>
   </si>
   <si>
-    <t>Prehab -24 (6)
-Control -10 (2)</t>
-  </si>
-  <si>
     <t>Control group- received standard hospital care</t>
   </si>
   <si>
@@ -421,10 +413,6 @@
   </si>
   <si>
     <t>Control group-  received usual clinical care</t>
-  </si>
-  <si>
-    <t>Prehabilitation – 18 (6) 
-Control – 22 (2)</t>
   </si>
   <si>
     <t>control group -received standard care which consisted of nutritional counseling, physical activity recommendations, and advice on smoking cessation</t>
@@ -648,10 +636,6 @@
 medical coaching adherence - 82 ± 20%</t>
   </si>
   <si>
-    <t>Prehabilitation – 52 (14) 
-Rehabilitation – 43 (15)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Multimodal program:
 1. Exercise: Home-based, unsupervised. Moderate-vigorous aerobic training for 30 minutes, 3 days/week. Resistance training with 10 exercises targeting major muscle groups, 2 sets of 8–12 repetitions, 3 days/week using elastic bands.
 2. Nutritional support: Individualized care from a registered dietitian. Target protein intake of 1.5 g/kg ideal body weight, supplemented with whey protein within 1 hour of exercise as needed.
@@ -868,6 +852,22 @@
   <si>
     <t>Nutrition -93.2%
 Exercises- 88.2% (home-based) and 84.1% (supervised)</t>
+  </si>
+  <si>
+    <t>Prehabilitation – 66 (14) 
+Rehabilitation – 58 (15)</t>
+  </si>
+  <si>
+    <t>Prehabilitation – 24(6)
+Control – 24 (2)</t>
+  </si>
+  <si>
+    <t>PREHAB+ - 41 (4)
+REHAB - 39 (13)</t>
+  </si>
+  <si>
+    <t>Prehab -24 (10)
+Control -10 (3)</t>
   </si>
 </sst>
 </file>
@@ -1407,7 +1407,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -1425,31 +1425,31 @@
         <v>1</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>71</v>
@@ -1461,25 +1461,25 @@
         <v>2</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>72</v>
@@ -1507,7 +1507,7 @@
         <v>74</v>
       </c>
       <c r="G2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>69</v>
@@ -1519,7 +1519,7 @@
         <v>3</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>3</v>
@@ -1528,43 +1528,43 @@
         <v>3</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q2" s="6" t="s">
         <v>75</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V2" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z2" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="AA2" s="22">
         <v>0.63</v>
@@ -1589,10 +1589,10 @@
         <v>22</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>78</v>
+        <v>240</v>
       </c>
       <c r="G3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>77</v>
@@ -1604,7 +1604,7 @@
         <v>3</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>3</v>
@@ -1613,46 +1613,46 @@
         <v>3</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q3" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA3" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="AB3" s="4"/>
       <c r="AC3" s="4"/>
@@ -1674,70 +1674,70 @@
         <v>8</v>
       </c>
       <c r="F4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" t="s">
+        <v>148</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="G4" t="s">
-        <v>151</v>
-      </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="4" t="s">
+      <c r="R4" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="X4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA4" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="R4" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="S4" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="T4" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="U4" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="W4" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="X4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y4" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="Z4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA4" s="4" t="s">
-        <v>84</v>
       </c>
       <c r="AB4" s="6"/>
       <c r="AC4" s="6"/>
@@ -1759,70 +1759,70 @@
         <v>8</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="R5" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W5" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X5" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z5" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AB5" s="4"/>
       <c r="AC5" s="4"/>
@@ -1835,19 +1835,19 @@
         <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>89</v>
+        <v>241</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
@@ -1859,7 +1859,7 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>3</v>
@@ -1868,7 +1868,7 @@
         <v>3</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>3</v>
@@ -1877,37 +1877,37 @@
         <v>3</v>
       </c>
       <c r="Q6" s="16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Z6" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA6" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="AB6" s="4"/>
       <c r="AC6" s="4"/>
@@ -1929,10 +1929,10 @@
         <v>8</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>20</v>
@@ -1944,7 +1944,7 @@
         <v>3</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>3</v>
@@ -1953,7 +1953,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O7" s="9" t="s">
         <v>3</v>
@@ -1962,37 +1962,37 @@
         <v>3</v>
       </c>
       <c r="Q7" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="S7" s="8" t="s">
         <v>21</v>
       </c>
       <c r="T7" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="U7" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V7" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="W7" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X7" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Y7" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Z7" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA7" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="AB7" s="4"/>
       <c r="AC7" s="4"/>
@@ -2014,10 +2014,10 @@
         <v>22</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>25</v>
@@ -2041,43 +2041,43 @@
         <v>3</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P8" s="5" t="s">
         <v>3</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
@@ -2099,10 +2099,10 @@
         <v>22</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>40</v>
@@ -2123,46 +2123,46 @@
         <v>3</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="T9" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W9" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X9" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Z9" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA9" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="AB9" s="4"/>
       <c r="AC9" s="4"/>
@@ -2184,10 +2184,10 @@
         <v>22</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>105</v>
+        <v>239</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>42</v>
@@ -2202,7 +2202,7 @@
         <v>3</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>3</v>
@@ -2214,40 +2214,40 @@
         <v>3</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="T10" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V10" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W10" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X10" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y10" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z10" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA10" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AB10" s="4"/>
       <c r="AC10" s="4"/>
@@ -2269,10 +2269,10 @@
         <v>22</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>43</v>
@@ -2284,7 +2284,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>3</v>
@@ -2293,43 +2293,43 @@
         <v>3</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W11" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X11" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y11" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Z11" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA11" s="23">
         <v>0.83299999999999996</v>
@@ -2354,10 +2354,10 @@
         <v>22</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>45</v>
@@ -2387,37 +2387,37 @@
         <v>3</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="T12" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W12" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AB12" s="4"/>
       <c r="AC12" s="4"/>
@@ -2439,10 +2439,10 @@
         <v>22</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>47</v>
@@ -2454,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>3</v>
@@ -2463,46 +2463,46 @@
         <v>3</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>3</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="T13" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="V13" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W13" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y13" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z13" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA13" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="AB13" s="4"/>
       <c r="AC13" s="5"/>
@@ -2524,10 +2524,10 @@
         <v>49</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G14" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>50</v>
@@ -2539,55 +2539,55 @@
         <v>3</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P14" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="T14" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="W14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="X14" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Y14" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA14" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="AB14" s="4"/>
       <c r="AC14" s="4"/>
@@ -2609,10 +2609,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>52</v>
@@ -2636,40 +2636,40 @@
         <v>3</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P15" s="5" t="s">
         <v>3</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="T15" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="U15" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V15" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="W15" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="X15" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y15" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z15" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA15" s="24">
         <v>0.873</v>
@@ -2694,10 +2694,10 @@
         <v>22</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>53</v>
@@ -2709,10 +2709,10 @@
         <v>3</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>3</v>
@@ -2727,34 +2727,34 @@
         <v>3</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="T16" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z16" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AA16" s="23">
         <v>0.84399999999999997</v>
@@ -2779,10 +2779,10 @@
         <v>22</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>55</v>
@@ -2794,7 +2794,7 @@
         <v>3</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L17" s="9" t="s">
         <v>3</v>
@@ -2809,40 +2809,40 @@
         <v>3</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="U17" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X17" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y17" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z17" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA17" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="AB17" s="4"/>
       <c r="AC17" s="4"/>
@@ -2864,10 +2864,10 @@
         <v>22</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G18" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>57</v>
@@ -2879,7 +2879,7 @@
         <v>3</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L18" s="4" t="s">
         <v>3</v>
@@ -2891,43 +2891,43 @@
         <v>3</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="R18" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="T18" s="4" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="U18" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V18" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W18" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X18" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y18" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z18" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="AA18" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="AB18" s="4"/>
       <c r="AC18" s="4"/>
@@ -2949,10 +2949,10 @@
         <v>22</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G19" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>59</v>
@@ -2964,55 +2964,55 @@
         <v>3</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L19" s="4" t="s">
         <v>3</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="T19" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="U19" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="V19" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W19" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X19" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y19" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z19" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA19" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="AB19" s="4"/>
       <c r="AC19" s="4"/>
@@ -3034,10 +3034,10 @@
         <v>22</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G20" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>61</v>
@@ -3046,7 +3046,7 @@
         <v>3</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>3</v>
@@ -3061,43 +3061,43 @@
         <v>3</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q20" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="T20" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U20" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V20" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="W20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="X20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y20" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AB20" s="4"/>
       <c r="AC20" s="4"/>
@@ -3119,10 +3119,10 @@
         <v>22</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>63</v>
@@ -3131,7 +3131,7 @@
         <v>3</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>3</v>
@@ -3146,43 +3146,43 @@
         <v>3</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P21" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="T21" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V21" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W21" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="X21" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y21" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z21" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA21" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="AB21" s="4"/>
       <c r="AC21" s="4"/>
@@ -3204,10 +3204,10 @@
         <v>66</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>67</v>
@@ -3219,55 +3219,55 @@
         <v>3</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="M22" s="5" t="s">
         <v>3</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P22" s="5" t="s">
         <v>3</v>
       </c>
       <c r="Q22" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="R22" s="5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="T22" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U22" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V22" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="W22" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="X22" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Y22" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z22" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA22" s="4" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="AB22" s="5"/>
       <c r="AC22" s="4"/>
@@ -3280,7 +3280,7 @@
         <v>15</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>68</v>
@@ -3289,13 +3289,13 @@
         <v>22</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>172</v>
+        <v>238</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>3</v>
@@ -3304,7 +3304,7 @@
         <v>3</v>
       </c>
       <c r="K23" s="20" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L23" s="20" t="s">
         <v>3</v>
@@ -3313,46 +3313,46 @@
         <v>3</v>
       </c>
       <c r="N23" s="20" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O23" s="20" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P23" s="20" t="s">
         <v>3</v>
       </c>
       <c r="Q23" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="R23" s="21" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="T23" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="U23" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="V23" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W23" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X23" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y23" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z23" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA23" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
@@ -3362,25 +3362,25 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C24" s="3">
         <v>2022</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>3</v>
@@ -3389,55 +3389,55 @@
         <v>3</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="M24" s="4" t="s">
         <v>3</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="P24" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="T24" s="4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="U24" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="V24" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="W24" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X24" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Y24" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="Z24" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AA24" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
@@ -3447,82 +3447,82 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C25" s="3">
         <v>2024</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F25" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="N25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="O25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="P25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q25" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="R25" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="S25" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="U25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="V25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W25" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="X25" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y25" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z25" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA25" s="5" t="s">
         <v>164</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="O25" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="P25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q25" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="R25" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="S25" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="T25" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="U25" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="V25" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="W25" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="X25" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y25" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="Z25" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA25" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>

</xml_diff>

<commit_message>
update evidence table and clean_data
</commit_message>
<xml_diff>
--- a/data/Evidence_Table.xlsx
+++ b/data/Evidence_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saramanaye/Documents/GitHub/cancer_nutrition_evidence_review/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BF9A19-CD80-8D40-AD89-B252DEBFB24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D4EA6D-3C83-D547-88D6-0E96CD8D965E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="14600" windowHeight="16140" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="14600" windowHeight="16120" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Table" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="241">
   <si>
     <t>Year</t>
   </si>
@@ -282,9 +282,6 @@
     <t>Waller et al.</t>
   </si>
   <si>
-    <t>Randomised controlled pilot study</t>
-  </si>
-  <si>
     <t>Tri-modal prehabilitation delivered via Fitbit smartwatch and smartphone apps:
 1. Exercise - Individualised aerobic exercise (3x/week) + resistance training with bands (2x/week) + 30 min of additional physical activity like walking or stairs (2x/week). Intensity tailored to 50–70% of predicted maximum heart rate and BORG scale 12–16.
 2. Nutrition - Written dietary advice and educational presentation focused on protein intake and avoiding weight loss + monitoring via Fitbit App food log.
@@ -725,9 +722,6 @@
 Psychological health</t>
   </si>
   <si>
-    <t>Randomized Controlled Feasibility Trial</t>
-  </si>
-  <si>
     <t>Author</t>
   </si>
   <si>
@@ -868,6 +862,9 @@
   <si>
     <t>Prehab -24 (10)
 Control -10 (3)</t>
+  </si>
+  <si>
+    <t>Pilot Randomised Controlled  Study</t>
   </si>
 </sst>
 </file>
@@ -1380,7 +1377,8 @@
     <col min="2" max="2" width="12.5" style="3" customWidth="1"/>
     <col min="3" max="3" width="19.33203125" customWidth="1"/>
     <col min="4" max="4" width="37" style="6" customWidth="1"/>
-    <col min="5" max="6" width="22.5" customWidth="1"/>
+    <col min="5" max="5" width="32.5" customWidth="1"/>
+    <col min="6" max="6" width="22.5" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="54.83203125" style="6" customWidth="1"/>
     <col min="9" max="9" width="25" style="6" customWidth="1"/>
@@ -1407,7 +1405,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -1416,73 +1414,73 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="L1" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="K1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>144</v>
-      </c>
       <c r="M1" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>147</v>
-      </c>
       <c r="Z1" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
@@ -1504,67 +1502,67 @@
         <v>8</v>
       </c>
       <c r="F2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q2" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="P2" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>75</v>
-      </c>
       <c r="R2" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V2" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Z2" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AA2" s="22">
         <v>0.63</v>
@@ -1589,70 +1587,70 @@
         <v>22</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="G3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q3" s="6" t="s">
+      <c r="R3" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA3" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>79</v>
       </c>
       <c r="AB3" s="4"/>
       <c r="AC3" s="4"/>
@@ -1674,70 +1672,70 @@
         <v>8</v>
       </c>
       <c r="F4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" t="s">
+        <v>147</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="G4" t="s">
-        <v>148</v>
-      </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="4" t="s">
+      <c r="R4" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="X4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA4" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="R4" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="S4" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="T4" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="U4" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="W4" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="X4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y4" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="Z4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA4" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="AB4" s="6"/>
       <c r="AC4" s="6"/>
@@ -1759,70 +1757,70 @@
         <v>8</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="R5" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W5" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X5" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z5" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB5" s="4"/>
       <c r="AC5" s="4"/>
@@ -1835,19 +1833,19 @@
         <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>196</v>
+        <v>165</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
@@ -1859,7 +1857,7 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>3</v>
@@ -1868,7 +1866,7 @@
         <v>3</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>3</v>
@@ -1877,37 +1875,37 @@
         <v>3</v>
       </c>
       <c r="Q6" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z6" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA6" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="AB6" s="4"/>
       <c r="AC6" s="4"/>
@@ -1929,10 +1927,10 @@
         <v>8</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>20</v>
@@ -1944,7 +1942,7 @@
         <v>3</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>3</v>
@@ -1953,7 +1951,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O7" s="9" t="s">
         <v>3</v>
@@ -1962,37 +1960,37 @@
         <v>3</v>
       </c>
       <c r="Q7" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="S7" s="8" t="s">
         <v>21</v>
       </c>
       <c r="T7" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="U7" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V7" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W7" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X7" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Y7" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z7" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA7" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AB7" s="4"/>
       <c r="AC7" s="4"/>
@@ -2014,10 +2012,10 @@
         <v>22</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>25</v>
@@ -2041,43 +2039,43 @@
         <v>3</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P8" s="5" t="s">
         <v>3</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
@@ -2099,10 +2097,10 @@
         <v>22</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>40</v>
@@ -2123,46 +2121,46 @@
         <v>3</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="T9" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W9" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X9" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z9" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA9" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AB9" s="4"/>
       <c r="AC9" s="4"/>
@@ -2184,10 +2182,10 @@
         <v>22</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>42</v>
@@ -2202,7 +2200,7 @@
         <v>3</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>3</v>
@@ -2214,40 +2212,40 @@
         <v>3</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="T10" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V10" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W10" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Z10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB10" s="4"/>
       <c r="AC10" s="4"/>
@@ -2269,10 +2267,10 @@
         <v>22</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>43</v>
@@ -2284,7 +2282,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>3</v>
@@ -2293,43 +2291,43 @@
         <v>3</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q11" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="R11" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="R11" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="S11" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W11" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X11" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y11" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z11" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA11" s="23">
         <v>0.83299999999999996</v>
@@ -2351,13 +2349,13 @@
         <v>30</v>
       </c>
       <c r="E12" t="s">
-        <v>22</v>
+        <v>165</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>45</v>
@@ -2387,37 +2385,37 @@
         <v>3</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="T12" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W12" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y12" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA12" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB12" s="4"/>
       <c r="AC12" s="4"/>
@@ -2439,10 +2437,10 @@
         <v>22</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>47</v>
@@ -2454,7 +2452,7 @@
         <v>3</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>3</v>
@@ -2463,46 +2461,46 @@
         <v>3</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>3</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="R13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="R13" s="6" t="s">
+      <c r="S13" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="V13" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W13" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Y13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA13" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="S13" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="T13" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="U13" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="V13" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W13" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X13" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Y13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA13" s="4" t="s">
-        <v>113</v>
       </c>
       <c r="AB13" s="4"/>
       <c r="AC13" s="5"/>
@@ -2524,10 +2522,10 @@
         <v>49</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>50</v>
@@ -2539,55 +2537,55 @@
         <v>3</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P14" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="T14" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="U14" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="W14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA14" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="R14" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="S14" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="T14" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="U14" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="W14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="X14" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="Y14" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA14" s="4" t="s">
-        <v>116</v>
       </c>
       <c r="AB14" s="4"/>
       <c r="AC14" s="4"/>
@@ -2609,10 +2607,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>52</v>
@@ -2636,40 +2634,40 @@
         <v>3</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P15" s="5" t="s">
         <v>3</v>
       </c>
       <c r="Q15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="R15" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="R15" s="5" t="s">
-        <v>119</v>
-      </c>
       <c r="S15" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="T15" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U15" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V15" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W15" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="X15" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Y15" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z15" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA15" s="24">
         <v>0.873</v>
@@ -2694,10 +2692,10 @@
         <v>22</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>53</v>
@@ -2709,10 +2707,10 @@
         <v>3</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>3</v>
@@ -2727,34 +2725,34 @@
         <v>3</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="T16" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z16" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AA16" s="23">
         <v>0.84399999999999997</v>
@@ -2779,10 +2777,10 @@
         <v>22</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>55</v>
@@ -2794,7 +2792,7 @@
         <v>3</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L17" s="9" t="s">
         <v>3</v>
@@ -2809,40 +2807,40 @@
         <v>3</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="U17" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X17" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Y17" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Z17" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA17" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AB17" s="4"/>
       <c r="AC17" s="4"/>
@@ -2864,10 +2862,10 @@
         <v>22</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>57</v>
@@ -2879,7 +2877,7 @@
         <v>3</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L18" s="4" t="s">
         <v>3</v>
@@ -2891,43 +2889,43 @@
         <v>3</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q18" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="R18" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="R18" s="4" t="s">
+      <c r="S18" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="T18" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="U18" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X18" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="AA18" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="T18" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="U18" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V18" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W18" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X18" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Y18" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z18" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="AA18" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="AB18" s="4"/>
       <c r="AC18" s="4"/>
@@ -2949,10 +2947,10 @@
         <v>22</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>59</v>
@@ -2964,55 +2962,55 @@
         <v>3</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L19" s="4" t="s">
         <v>3</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q19" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="U19" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="V19" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W19" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Y19" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z19" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA19" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="R19" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="S19" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="T19" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="U19" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="V19" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W19" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X19" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Y19" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z19" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA19" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="AB19" s="4"/>
       <c r="AC19" s="4"/>
@@ -3034,10 +3032,10 @@
         <v>22</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>61</v>
@@ -3046,7 +3044,7 @@
         <v>3</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>3</v>
@@ -3061,43 +3059,43 @@
         <v>3</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q20" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="T20" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U20" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V20" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="X20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y20" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB20" s="4"/>
       <c r="AC20" s="4"/>
@@ -3119,10 +3117,10 @@
         <v>22</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G21" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>63</v>
@@ -3131,7 +3129,7 @@
         <v>3</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>3</v>
@@ -3146,43 +3144,43 @@
         <v>3</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P21" s="6" t="s">
         <v>3</v>
       </c>
       <c r="Q21" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="R21" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="R21" s="6" t="s">
+      <c r="S21" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="U21" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V21" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W21" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA21" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="S21" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="T21" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="U21" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V21" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W21" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="X21" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y21" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z21" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA21" s="4" t="s">
-        <v>136</v>
       </c>
       <c r="AB21" s="4"/>
       <c r="AC21" s="4"/>
@@ -3201,73 +3199,73 @@
         <v>64</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="I22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="N22" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="O22" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="P22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q22" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="N22" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="O22" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="P22" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q22" s="4" t="s">
+      <c r="R22" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="S22" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="T22" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="U22" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="W22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="X22" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA22" s="4" t="s">
         <v>172</v>
-      </c>
-      <c r="R22" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="S22" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="T22" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="U22" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="W22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="X22" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="Y22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA22" s="4" t="s">
-        <v>173</v>
       </c>
       <c r="AB22" s="5"/>
       <c r="AC22" s="4"/>
@@ -3280,79 +3278,79 @@
         <v>15</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H23" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J23" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K23" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="L23" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="N23" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="O23" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="P23" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q23" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="R23" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="S23" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="U23" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W23" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y23" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA23" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="K23" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="L23" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="N23" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="O23" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="P23" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q23" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="R23" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="S23" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="T23" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="U23" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="V23" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W23" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X23" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y23" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z23" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA23" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
@@ -3362,82 +3360,82 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C24" s="3">
         <v>2022</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E24" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H24" s="4" t="s">
+      <c r="I24" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="P24" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="R24" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="S24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="T24" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="U24" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V24" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="W24" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X24" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Y24" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z24" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA24" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="N24" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="O24" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P24" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q24" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="R24" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="S24" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="T24" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="U24" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V24" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="W24" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X24" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Y24" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z24" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="AA24" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
@@ -3447,82 +3445,82 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C25" s="3">
         <v>2024</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F25" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H25" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="H25" s="5" t="s">
+      <c r="I25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="N25" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="O25" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="P25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q25" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="R25" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="S25" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="I25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="O25" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="P25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q25" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="R25" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="S25" s="4" t="s">
+      <c r="T25" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="U25" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="V25" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="W25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="X25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA25" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="T25" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="U25" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="V25" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="W25" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="X25" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y25" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="Z25" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA25" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>

</xml_diff>

<commit_message>
year updates in evidence table
</commit_message>
<xml_diff>
--- a/data/Evidence_Table.xlsx
+++ b/data/Evidence_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saramanaye/Documents/GitHub/cancer_nutrition_evidence_review/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D4EA6D-3C83-D547-88D6-0E96CD8D965E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47F7C08-6335-BA4F-8A26-00466FFFC647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="14600" windowHeight="16120" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{4D926D7D-19DF-E54A-9976-ED1795FE3A18}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Table" sheetId="1" r:id="rId1"/>
@@ -2768,7 +2768,7 @@
         <v>54</v>
       </c>
       <c r="C17">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>35</v>
@@ -2853,7 +2853,7 @@
         <v>56</v>
       </c>
       <c r="C18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>36</v>

</xml_diff>